<commit_message>
Dashboard update: Avance de cronograma actualizado vía API
</commit_message>
<xml_diff>
--- a/Cronograma_Fase2_ABA.xlsx
+++ b/Cronograma_Fase2_ABA.xlsx
@@ -461,10 +461,10 @@
         <v>2026-05-15</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J2" t="str">
-        <v>Completado</v>
+        <v>En progreso</v>
       </c>
       <c r="K2" t="str">
         <v/>
@@ -496,10 +496,10 @@
         <v>2026-05-15</v>
       </c>
       <c r="I3">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="J3" t="str">
-        <v>En progreso</v>
+        <v>Completado</v>
       </c>
       <c r="K3" t="str">
         <v/>

</xml_diff>